<commit_message>
Implementado novos campos no modelo e refinado tradeBot
</commit_message>
<xml_diff>
--- a/Rodovias/modelos_rodovias/doutor_manoel_hyppolito_rego_km_83_caraguatatuba_sp_rf_regimes/importancias.xlsx
+++ b/Rodovias/modelos_rodovias/doutor_manoel_hyppolito_rego_km_83_caraguatatuba_sp_rf_regimes/importancias.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,370 +431,470 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>meta_num</t>
+          <t>roll5_ratio_pass_total_meta</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.09829358085180215</v>
+        <v>0.07478174828331491</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>interacao_meta_temperatura</t>
+          <t>roll3_ratio_pass_total_meta</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.09448755956690379</v>
+        <v>0.06877069125199312</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>interacao_meta_umidade</t>
+          <t>meta_num</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.09228907840792358</v>
+        <v>0.0523131147480474</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>interacao_meta_hora_cos</t>
+          <t>interacao_meta_umidade</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.08498211063531623</v>
+        <v>0.05001052203140716</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>interacao_meta_hora_sin</t>
+          <t>interacao_meta_temperatura</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.08104446602590142</v>
+        <v>0.04953845918597775</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>minuto</t>
+          <t>lag1_ratio_pass_total_meta</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.07655497001564021</v>
+        <v>0.04454521510561107</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>hora_decimal</t>
+          <t>minuto</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.06546405409704271</v>
+        <v>0.04318562445092283</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>hora_sin</t>
+          <t>lag1_pass_total_mercado</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.06464564270105029</v>
+        <v>0.04252582867774504</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>hora_cos</t>
+          <t>interacao_meta_hora_sin</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.06223985705573378</v>
+        <v>0.04180752741765491</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>temperatura_2m</t>
+          <t>roll10_mean_pass_total_mercado</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.04553602950644316</v>
+        <v>0.04142976384251271</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>umidade_relativa</t>
+          <t>lag1_pass_tendencia_5m</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04481199826683947</v>
+        <v>0.04111567860631542</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cobertura_nuvens</t>
+          <t>roll3_mean_pass_total_mercado</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.04328400644212667</v>
+        <v>0.04067060922020103</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dia_semana_sin</t>
+          <t>interacao_meta_hora_cos</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.02546418942697824</v>
+        <v>0.04018799808175542</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>dia_semana</t>
+          <t>roll5_mean_pass_total_mercado</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.02221255917969205</v>
+        <v>0.03933008363604673</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>hora_decimal</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.01731402808847468</v>
+        <v>0.03453449876612519</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>dia_semana_cos</t>
+          <t>hora_sin</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.01475276748651875</v>
+        <v>0.03439347685767766</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>chuva_mm</t>
+          <t>hora_cos</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.01342335828778472</v>
+        <v>0.03388183668659462</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>bloco_dia_cod</t>
+          <t>lag1_pass_qtd_ultimos_2min</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.006256575372993039</v>
+        <v>0.03029789867542981</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>eh_sexta</t>
+          <t>lag1_pass_media_ultimos_2min</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.00619208965720662</v>
+        <v>0.02978521010371921</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>estava_chovendo</t>
+          <t>temperatura_2m</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.004536049025572631</v>
+        <v>0.02660508470769219</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>eh_dia_util</t>
+          <t>umidade_relativa</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.004286935478496083</v>
+        <v>0.02516139938927648</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>fim_semana</t>
+          <t>cobertura_nuvens</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.003930399737755038</v>
+        <v>0.02483643518637903</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>eh_sabado</t>
+          <t>dia_semana</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.003748621173985256</v>
+        <v>0.01379007333120661</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>bloco_manha</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.003576445515269794</v>
+        <v>0.01285961639629494</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>eh_domingo</t>
+          <t>dia_semana_sin</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.003265898433676692</v>
+        <v>0.01249017595868819</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>bloco_almoco</t>
+          <t>dia_semana_cos</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.003030975681744054</v>
+        <v>0.00930675911970026</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>eh_pico_tarde</t>
+          <t>chuva_mm</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.002443489869397214</v>
+        <v>0.008104353339286807</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>bloco_tarde_pico</t>
+          <t>bloco_dia_cod</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.002399421383950762</v>
+        <v>0.004942324866135829</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>eh_pico_manha</t>
+          <t>bloco_manha</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.002202364045053316</v>
+        <v>0.003075498442985815</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>mes_cos</t>
+          <t>eh_sexta</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.001816951628267528</v>
+        <v>0.002890536201874449</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>bloco_pico_manha</t>
+          <t>estava_chovendo</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.001757048121337187</v>
+        <v>0.002559368965892924</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>mes_sin</t>
+          <t>bloco_almoco</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.001652921853221685</v>
+        <v>0.002513225363622032</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>mes</t>
+          <t>eh_pico_tarde</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.001652355049690936</v>
+        <v>0.002378580882357496</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>bloco_noite</t>
+          <t>eh_sabado</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.0004512019302102771</v>
+        <v>0.002241609093000196</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>bloco_madrugada</t>
+          <t>eh_dia_util</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0</v>
+        <v>0.002141461618254904</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>bloco_outro</t>
+          <t>fim_semana</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0</v>
+        <v>0.002053899892863</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>bloco_tarde_pico</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0.001661823422085115</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>eh_pico_manha</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.001606671732546347</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>eh_domingo</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0.001274064344998207</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>bloco_pico_manha</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0.001135849222020959</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>mes_cos</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0.001043671129022276</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>mes_sin</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0.0009958900896594374</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0.0009252627723412648</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>bloco_noite</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0.000300578902763317</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>bloco_madrugada</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>bloco_outro</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>bloco_late_night</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B48" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>